<commit_message>
feat(cv-cli): add AVIF image conversion routes and test fixtures
</commit_message>
<xml_diff>
--- a/packages/cv-cli/test/fixtures/input.xlsx
+++ b/packages/cv-cli/test/fixtures/input.xlsx
@@ -124,37 +124,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -254,8 +254,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>